<commit_message>
now it is more polished and supports using KPI name and not kpiid
now it is more polished and supports using KPI name and not kpiid
</commit_message>
<xml_diff>
--- a/excel/HDA heatmap example.xlsx
+++ b/excel/HDA heatmap example.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luca.paone\github\PTV-Flows-tutorials\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptvgroup-my.sharepoint.com/personal/luca_paone_ptvgroup_com/Documents/Documents/GitHub/PTV-Mobility/PTV-Flows-tutorials/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{415C5598-6086-47C6-A4E5-D02301BE4A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{415C5598-6086-47C6-A4E5-D02301BE4A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F933E2A-D665-4059-88F3-52B41FCE10A6}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="57">
   <si>
     <t>apiKey &gt;</t>
   </si>
@@ -92,15 +92,6 @@
     <t>Location ID</t>
   </si>
   <si>
-    <t>you can use the TomTom demo  decoder at https://demo.tomtom.com/  to check the position of the OpenLR code</t>
-  </si>
-  <si>
-    <t>you can use https://geohashviz.com/  to visualize the geohash to be used inside HAD</t>
-  </si>
-  <si>
-    <t>2025-01-17T00:00:28Z</t>
-  </si>
-  <si>
     <t xml:space="preserve">&lt; apiKey </t>
   </si>
   <si>
@@ -116,14 +107,138 @@
     <t>DAYS_1</t>
   </si>
   <si>
-    <t>2025-01-31T23:59:28Z</t>
+    <t>KPI NAME
+ (copy from the KPI table below)</t>
+  </si>
+  <si>
+    <t>2025-01-30T23:59:28Z</t>
+  </si>
+  <si>
+    <t>Datetime</t>
+  </si>
+  <si>
+    <t>Request URL</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>2025-02-21T12:18:37.672Z</t>
+  </si>
+  <si>
+    <t>https://api.ptvgroup.tech/kpieng/v1/instance/all</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>2025-02-21T12:29:42.360Z</t>
+  </si>
+  <si>
+    <t>https://api.ptvgroup.tech/hda/v1/kpi/overall/get?kpiId=b141a34f-ae17-4ea2-bea5-5ee50a112659&amp;fromTime=2025-01-30T23%3A59%3A28Z&amp;toTime=2025-01-31T23%3A59%3A28Z&amp;timeAggregation=MINUTES_5</t>
+  </si>
+  <si>
+    <t>2025-01-31T03:59:28Z</t>
+  </si>
+  <si>
+    <t>2025-02-21T12:34:15.132Z</t>
+  </si>
+  <si>
+    <t>https://api.ptvgroup.tech/hda/v1/kpi/detailed/get?kpiId=b141a34f-ae17-4ea2-bea5-5ee50a112659&amp;fromTime=2025-01-30T23%3A59%3A28Z&amp;toTime=2025-01-31T03%3A59%3A28Z&amp;timeAggregation=MINUTES_5</t>
+  </si>
+  <si>
+    <t>Create an API key from your PTV Flows instance and copy it into the Config tab, cell B1.</t>
+  </si>
+  <si>
+    <t>Select the From and To dates in cells B3 and C3 respectively.</t>
+  </si>
+  <si>
+    <t>Create the heatmap for the detailed results.</t>
+  </si>
+  <si>
+    <t>NOTE:</t>
+  </si>
+  <si>
+    <t>You can use https://geohashviz.com/ to visualize the geohash to be used inside HAD.</t>
+  </si>
+  <si>
+    <t>You can use the TomTom demo decoder at https://demo.tomtom.com/ to check the position of the OpenLR code.</t>
+  </si>
+  <si>
+    <t>By following these steps:</t>
+  </si>
+  <si>
+    <t>Date Format: Dates must be in ISO 8601 format to be correctly processed by the scripts and API.</t>
+  </si>
+  <si>
+    <t>README</t>
+  </si>
+  <si>
+    <t>Click on the "Get KPI Definitions" button.</t>
+  </si>
+  <si>
+    <t>This will retrieve the list of available KPIs and populate the KPI_list table with their IDs, names, and associated locations.</t>
+  </si>
+  <si>
+    <t>In the Config tab, cell A3, enter the name of the KPI from which you want to get the data.</t>
+  </si>
+  <si>
+    <t>Ensure that the KPI name matches exactly as listed in the KPI_list table.</t>
+  </si>
+  <si>
+    <t>Dates should be in ISO 8601 format (e.g., 2023-01-01T00:00:00Z).</t>
+  </si>
+  <si>
+    <t>The From date must be before the To date.</t>
+  </si>
+  <si>
+    <t>For the "Detailed Results" button, the time interval between From and To should not exceed 24 hours.</t>
+  </si>
+  <si>
+    <t>Download the data by clicking on the "KPI Overall Results" or "Detailed Results" buttons.</t>
+  </si>
+  <si>
+    <t>KPI Overall Results: Retrieves aggregated KPI data over the selected time range.</t>
+  </si>
+  <si>
+    <t>Detailed Results: Retrieves detailed KPI data within the selected time range.</t>
+  </si>
+  <si>
+    <t>OR create the pivot data for further analysis for the overall results.</t>
+  </si>
+  <si>
+    <t>API Key Setup: Place your API key in cell B1 of the Config tab to authenticate with the PTV Flows API.</t>
+  </si>
+  <si>
+    <t>Retrieving KPI Definitions: Clicking the "Get KPI Definitions" button will update the KPI_list table with current KPI information.</t>
+  </si>
+  <si>
+    <t>Selecting a KPI: Enter the KPI Name into cell A3. The scripts will automatically find the corresponding KPI ID from the KPI_list table.</t>
+  </si>
+  <si>
+    <t>Setting Date Range: Input your desired date range in cells B3 (From date) and C3 (To date), ensuring the dates are valid and in the correct format.</t>
+  </si>
+  <si>
+    <t>Downloading Data: Use the buttons provided to retrieve the data. Note that for detailed results, the date range should not exceed 24 hours.</t>
+  </si>
+  <si>
+    <t>Further Analysis: Proceed to create heatmaps or pivot tables as desired for your analysis.</t>
+  </si>
+  <si>
+    <t>Important Notes:</t>
+  </si>
+  <si>
+    <t>Time Aggregation (if applicable): Ensure that any time aggregation parameters are entered correctly in the appropriate cell (e.g., cell D3) with valid values like "MINUTES_5", "HOURS_1", etc.</t>
+  </si>
+  <si>
+    <t>Error Handling: If there are issues with your input (e.g., invalid dates, KPI Name not found), the scripts will provide error messages directly in the relevant cells or in a Log worksheet.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,8 +280,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -184,8 +307,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -223,35 +358,139 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF3F3F3F"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF3F3F3F"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF3F3F3F"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF3F3F3F"/>
+        </top>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -671,6 +910,31 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{177B2F8E-E2D6-4069-84DA-7D18928C2A9C}" name="KPI_list" displayName="KPI_list" ref="A14:D31" totalsRowShown="0" headerRowDxfId="6" dataDxfId="0" headerRowBorderDxfId="7" tableBorderDxfId="8" headerRowCellStyle="Output">
+  <autoFilter ref="A14:D31" xr:uid="{177B2F8E-E2D6-4069-84DA-7D18928C2A9C}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{C2E34D04-827E-4FE9-8555-F9759358324C}" name="KPI ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{15D7EBD1-93ED-48DD-8A6A-9A708CC5EC93}" name="KPI Name" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{4EF8EE06-C2A6-4326-A3A6-C47D75B236ED}" name="Location Name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{C03F7743-6F79-40D6-8DBB-10A1DB248141}" name="Location ID" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0199B611-4089-4C19-B903-690FA850BC44}" name="RequestLog" displayName="RequestLog" ref="A1:C4" totalsRowShown="0">
+  <autoFilter ref="A1:C4" xr:uid="{0199B611-4089-4C19-B903-690FA850BC44}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{29D2CF83-5A81-450A-8A89-B67A44631BC6}" name="Datetime"/>
+    <tableColumn id="2" xr3:uid="{D3409919-EAAA-404A-8A51-0EE86DFA49D2}" name="Request URL"/>
+    <tableColumn id="3" xr3:uid="{0953E0E5-637C-4436-91B0-0AECAA6BD877}" name="Status" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -934,7 +1198,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
@@ -953,34 +1217,34 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
+      <c r="B1" s="6"/>
       <c r="C1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="11" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="10" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>4</v>
       </c>
     </row>
@@ -989,87 +1253,380 @@
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>17</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E9" s="9"/>
+      <c r="E9" s="7"/>
     </row>
     <row r="10" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E10" s="5"/>
+      <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E11" s="3"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="12"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="13"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="12"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="12"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D3C5080-43A5-44C9-8422-A0ED9ADBB8E1}">
-  <dimension ref="C1"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" customWidth="1"/>
     <col min="2" max="2" width="57.42578125" customWidth="1"/>
     <col min="3" max="3" width="18.42578125" style="2" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD0D82FA-FD42-4D62-AAF4-10567937BF75}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
+      <c r="A1" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1078,17 +1635,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
+</scriptIds>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002632A3CB0C6CDD4EA758E3E5A84892AF" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c6c7bcb5e773f9f7da0ee88a749e050">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6" xmlns:ns3="43744f66-d8c7-4420-ad58-b4d72814d14f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ebd9547eaff2c58e2be891023bba85c" ns2:_="" ns3:_="">
     <xsd:import namespace="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
@@ -1317,43 +1882,35 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
-</scriptIds>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
+    <ds:schemaRef ds:uri=""/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E32AD742-8CF8-4A25-BDB4-C877FB6C5FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1372,19 +1929,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
-    <ds:schemaRef ds:uri=""/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>